<commit_message>
coa restructure and bug fix
</commit_message>
<xml_diff>
--- a/wwwroot/assets/doc_form/customer_upload_format.xlsx
+++ b/wwwroot/assets/doc_form/customer_upload_format.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iHishab\iHishab\wwwroot\assets\doc_form\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9CF097-6763-4CBB-8FB1-326E21425F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A36FCE-BA17-4663-9AF1-9E50495A30E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9754201E-3AEF-4F9D-85F1-81B96804210C}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9754201E-3AEF-4F9D-85F1-81B96804210C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Customer Name</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>Contact Mobile</t>
+  </si>
+  <si>
+    <t>NID</t>
   </si>
 </sst>
 </file>
@@ -477,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D370731B-2D29-4FB5-9410-F7697AB613E1}">
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
@@ -491,19 +494,20 @@
     <col min="9" max="9" width="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5.5546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="4.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.77734375" customWidth="1"/>
+    <col min="13" max="13" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="2" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="2" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -538,33 +542,36 @@
         <v>6</v>
       </c>
       <c r="L1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>